<commit_message>
no-mistakes(review): Sanitize private path from workbook metadata
</commit_message>
<xml_diff>
--- a/universal_mapping_schema.xlsx
+++ b/universal_mapping_schema.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sadoo\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{ECB31A83-8363-43AD-AF56-D7A0F099DCF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2472" yWindow="2472" windowWidth="17748" windowHeight="11736" activeTab="2" xr2:uid="{C2D3748E-272B-44A9-83DB-526D4E48591F}"/>

</xml_diff>

<commit_message>
Rename universal variable schema terms
</commit_message>
<xml_diff>
--- a/universal_mapping_schema.xlsx
+++ b/universal_mapping_schema.xlsx
@@ -8,7 +8,7 @@
     <workbookView xWindow="2472" yWindow="2472" windowWidth="17748" windowHeight="11736" activeTab="2" xr2:uid="{C2D3748E-272B-44A9-83DB-526D4E48591F}"/>
   </bookViews>
   <sheets>
-    <sheet name="universal_uid" sheetId="1" r:id="rId1"/>
+    <sheet name="universal_variable" sheetId="1" r:id="rId1"/>
     <sheet name="domain_variable" sheetId="2" r:id="rId2"/>
     <sheet name="estimation_template" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -44,7 +44,7 @@
     <t>datatype</t>
   </si>
   <si>
-    <t>context</t>
+    <t>description</t>
   </si>
   <si>
     <t>unit</t>
@@ -59,7 +59,7 @@
     <t>technology</t>
   </si>
   <si>
-    <t>variable_group</t>
+    <t>estimation_phase</t>
   </si>
   <si>
     <t>name</t>

</xml_diff>

<commit_message>
Add template domain variable bridge
</commit_message>
<xml_diff>
--- a/universal_mapping_schema.xlsx
+++ b/universal_mapping_schema.xlsx
@@ -11,6 +11,7 @@
     <sheet name="universal_variable" sheetId="1" r:id="rId1"/>
     <sheet name="domain_variable" sheetId="2" r:id="rId2"/>
     <sheet name="estimation_template" sheetId="3" r:id="rId3"/>
+    <sheet name="template_domain_variable" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1001,4 +1002,100 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>template_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>domain_uid</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>101</v>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>S_A_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>102</v>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>S_A_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>102</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>S_A_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>103</v>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>S_E_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>104</v>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>S_M_1_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>201</v>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>B_A_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>202</v>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>B_A_1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove universal variable domain UID list
</commit_message>
<xml_diff>
--- a/universal_mapping_schema.xlsx
+++ b/universal_mapping_schema.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
   <si>
     <t>universal_uid</t>
   </si>
@@ -54,9 +54,6 @@
     <t>domain_uid</t>
   </si>
   <si>
-    <t>domain_uid_list</t>
-  </si>
-  <si>
     <t>technology</t>
   </si>
   <si>
@@ -103,15 +100,6 @@
   </si>
   <si>
     <t>NULL</t>
-  </si>
-  <si>
-    <t>{S_A_1, B_A_1, W_A_1}</t>
-  </si>
-  <si>
-    <t>{S_A_2, B_A_2, W_A_2}</t>
-  </si>
-  <si>
-    <t>{S_A_3, B_A_3}</t>
   </si>
   <si>
     <t>S_A_1</t>
@@ -585,17 +573,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75C76BE5-4E70-4196-8D69-AC8A01834F14}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -608,59 +595,47 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -688,16 +663,16 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
-      </c>
-      <c r="F1" t="s">
-        <v>9</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -705,140 +680,140 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F2">
         <v>250</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
         <v>34</v>
-      </c>
-      <c r="E3" t="s">
-        <v>38</v>
       </c>
       <c r="F3">
         <v>180</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F4">
         <v>400</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F5">
         <v>30000</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B6">
         <v>7</v>
       </c>
       <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" t="s">
-        <v>35</v>
-      </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F6">
         <v>240</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B7">
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F7">
         <v>248</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -861,22 +836,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -884,19 +859,19 @@
         <v>101</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -904,19 +879,19 @@
         <v>102</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -924,19 +899,19 @@
         <v>103</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -944,19 +919,19 @@
         <v>104</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -964,19 +939,19 @@
         <v>201</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -984,19 +959,19 @@
         <v>202</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>